<commit_message>
Update proof generation scripts and experiment results
</commit_message>
<xml_diff>
--- a/Formal_Proof_Generation_Project/results/zero_shot_results.xlsx
+++ b/Formal_Proof_Generation_Project/results/zero_shot_results.xlsx
@@ -878,16 +878,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>51.52</v>
+        <v>30.3</v>
       </c>
       <c r="C3" t="n">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="D3" t="n">
-        <v>47.06</v>
+        <v>14.71</v>
       </c>
       <c r="E3" t="n">
-        <v>60.61</v>
+        <v>78.79000000000001</v>
       </c>
     </row>
     <row r="4"/>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>70.37</v>
+        <v>56.79</v>
       </c>
       <c r="C8" t="n">
-        <v>40</v>
+        <v>53.33</v>
       </c>
       <c r="D8" t="n">
-        <v>51.28</v>
+        <v>64.09999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>